<commit_message>
paper run 2026-10-02 10:05
</commit_message>
<xml_diff>
--- a/reports/2026-10-02.xlsx
+++ b/reports/2026-10-02.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,135 @@
       </c>
       <c r="K2" t="n">
         <v>108.61</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-02T04:58:17.216597+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F3" t="n">
+        <v>26.55</v>
+      </c>
+      <c r="G3" t="n">
+        <v>45</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00123</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>18.45</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-02T05:04:20.117217+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="F4" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>40</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.797</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00126</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-02T05:11:33.661909+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F5" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00186</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>10.5</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>108.61</v>
+        <v>153.76</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>108.61</v>
+        <v>153.76</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2667.429999999999</v>
+        <v>2712.579999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,329 +810,568 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>108.62</v>
+        <v>287.85</v>
       </c>
       <c r="E15" t="n">
-        <v>108.61</v>
+        <v>137.56</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>91.41</v>
+      </c>
+      <c r="E16" t="n">
+        <v>16.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>108.62</v>
-      </c>
-      <c r="E17" t="n">
-        <v>108.61</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>92.68000000000001</v>
+      </c>
+      <c r="E18" t="n">
+        <v>18.45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>108.62</v>
+        <v>189.25</v>
       </c>
       <c r="E19" t="n">
-        <v>108.61</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>97.33</v>
+      </c>
+      <c r="E20" t="n">
+        <v>108.61</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="n">
-        <v>108.62</v>
-      </c>
-      <c r="E21" t="n">
+          <t>По цене входа</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>224.15</v>
+      </c>
+      <c r="E22" t="n">
         <v>108.61</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>155.11</v>
+      </c>
+      <c r="E23" t="n">
+        <v>45.15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-11.29</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>108.61</v>
+        <v>390.55</v>
+      </c>
+      <c r="E26" t="n">
+        <v>153.76</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>108.61</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>18.45</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>108.61</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>108.61</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>137.56</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>108.61</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>108.61</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>18.45</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>108.61</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" t="n">
+        <v>45.15</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>108.61</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="n">
+        <v>34.65</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>108.61</v>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>127.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-02 17:40
</commit_message>
<xml_diff>
--- a/reports/2026-10-02.xlsx
+++ b/reports/2026-10-02.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,92 @@
       </c>
       <c r="K5" t="n">
         <v>10.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-02T12:41:16.391447+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>27.44</v>
+      </c>
+      <c r="G6" t="n">
+        <v>49</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.785</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>21.56</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-02T16:11:32.349347+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="G7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.00133</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>-10.98</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -699,7 +785,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -709,7 +795,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>153.76</v>
+        <v>164.34</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>153.76</v>
+        <v>175.32</v>
       </c>
     </row>
     <row r="8">
@@ -739,7 +825,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-10.98</v>
       </c>
     </row>
     <row r="9">
@@ -749,7 +835,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>15.97</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2712.579999999999</v>
+        <v>2723.159999999998</v>
       </c>
     </row>
     <row r="12">
@@ -810,16 +896,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>287.85</v>
+        <v>550.95</v>
       </c>
       <c r="E15" t="n">
-        <v>137.56</v>
+        <v>148.14</v>
       </c>
     </row>
     <row r="16">
@@ -829,13 +915,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>91.41</v>
+        <v>199.77</v>
       </c>
       <c r="E16" t="n">
         <v>16.2</v>
@@ -851,7 +937,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -861,297 +947,316 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>92.68000000000001</v>
+        <v>94.25</v>
       </c>
       <c r="E18" t="n">
-        <v>18.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>189.25</v>
+        <v>337.18</v>
       </c>
       <c r="E19" t="n">
-        <v>26.7</v>
+        <v>18.45</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>97.33</v>
+        <v>157.4</v>
       </c>
       <c r="E20" t="n">
-        <v>108.61</v>
+        <v>37.28</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>161.89</v>
+      </c>
+      <c r="E21" t="n">
+        <v>108.61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>2</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" t="n">
-        <v>224.15</v>
-      </c>
-      <c r="E22" t="n">
-        <v>108.61</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>155.11</v>
+        <v>702.2</v>
       </c>
       <c r="E23" t="n">
-        <v>45.15</v>
+        <v>108.61</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>226.01</v>
+      </c>
+      <c r="E24" t="n">
+        <v>66.70999999999999</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>-11.29</v>
+        <v>-177.49</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-10.98</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>4</v>
-      </c>
-      <c r="C26" t="n">
-        <v>4</v>
-      </c>
-      <c r="D26" t="n">
-        <v>390.55</v>
-      </c>
-      <c r="E26" t="n">
-        <v>153.76</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>344.63</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" t="n">
+        <v>25.63</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="n">
+        <v>380.46</v>
+      </c>
+      <c r="E29" t="n">
+        <v>164.34</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>18.45</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" t="n">
-        <v>26.7</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>108.61</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>18.45</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>37.28</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>137.56</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>16.2</v>
+        <v>108.61</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>148.14</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1161,216 +1266,318 @@
         <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>108.61</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>18.45</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" t="n">
-        <v>26.7</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>108.61</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>18.45</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" t="n">
-        <v>108.61</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>45.15</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>21.56</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-10.98</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" t="n">
-        <v>108.61</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>34.65</v>
+        <v>108.61</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D51" t="n">
-        <v>10.5</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>66.70999999999999</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-10.98</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="n">
-        <v>26.7</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>108.61</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>23.67</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>21.56</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D61" t="n">
+        <v>37.28</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B62" t="n">
         <v>2</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C62" t="n">
         <v>2</v>
       </c>
-      <c r="D55" t="n">
+      <c r="D62" t="n">
         <v>127.06</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-10-02 23:20
</commit_message>
<xml_diff>
--- a/reports/2026-10-02.xlsx
+++ b/reports/2026-10-02.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -730,6 +730,49 @@
       </c>
       <c r="K7" t="n">
         <v>-10.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-02T19:11:18.800080+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.00161</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>3.04</v>
       </c>
     </row>
   </sheetData>
@@ -743,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -765,7 +808,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -775,7 +818,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -795,7 +838,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="6">
@@ -805,7 +848,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>164.34</v>
+        <v>167.38</v>
       </c>
     </row>
     <row r="7">
@@ -815,7 +858,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>175.32</v>
+        <v>178.36</v>
       </c>
     </row>
     <row r="8">
@@ -835,7 +878,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15.97</v>
+        <v>16.24</v>
       </c>
     </row>
     <row r="10">
@@ -845,7 +888,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2723.159999999998</v>
+        <v>2726.199999999998</v>
       </c>
     </row>
     <row r="12">
@@ -896,16 +939,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>550.95</v>
+        <v>485.14</v>
       </c>
       <c r="E15" t="n">
-        <v>148.14</v>
+        <v>151.18</v>
       </c>
     </row>
     <row r="16">
@@ -915,13 +958,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>199.77</v>
+        <v>379.66</v>
       </c>
       <c r="E16" t="n">
         <v>16.2</v>
@@ -979,16 +1022,16 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
         <v>6</v>
       </c>
-      <c r="C20" t="n">
-        <v>4</v>
-      </c>
       <c r="D20" t="n">
-        <v>157.4</v>
+        <v>317.96</v>
       </c>
       <c r="E20" t="n">
-        <v>37.28</v>
+        <v>40.32</v>
       </c>
     </row>
     <row r="21">
@@ -998,13 +1041,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>161.89</v>
+        <v>115.41</v>
       </c>
       <c r="E21" t="n">
         <v>108.61</v>
@@ -1024,13 +1067,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
         <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>702.2</v>
+        <v>566.04</v>
       </c>
       <c r="E23" t="n">
         <v>108.61</v>
@@ -1043,13 +1086,13 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>9</v>
+      </c>
+      <c r="C24" t="n">
         <v>7</v>
       </c>
-      <c r="C24" t="n">
-        <v>5</v>
-      </c>
       <c r="D24" t="n">
-        <v>226.01</v>
+        <v>405.9</v>
       </c>
       <c r="E24" t="n">
         <v>66.70999999999999</v>
@@ -1062,16 +1105,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>-177.49</v>
+        <v>-107.14</v>
       </c>
       <c r="E25" t="n">
-        <v>-10.98</v>
+        <v>-7.94</v>
       </c>
     </row>
     <row r="26">
@@ -1088,13 +1131,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C27" t="n">
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>344.63</v>
+        <v>208.47</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1107,13 +1150,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>25.63</v>
+        <v>205.52</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1126,16 +1169,16 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" t="n">
         <v>6</v>
       </c>
-      <c r="C29" t="n">
-        <v>5</v>
-      </c>
       <c r="D29" t="n">
-        <v>380.46</v>
+        <v>450.81</v>
       </c>
       <c r="E29" t="n">
-        <v>164.34</v>
+        <v>167.38</v>
       </c>
     </row>
     <row r="31">
@@ -1190,13 +1233,13 @@
         </is>
       </c>
       <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" t="n">
         <v>4</v>
       </c>
-      <c r="C35" t="n">
-        <v>3</v>
-      </c>
       <c r="D35" t="n">
-        <v>37.28</v>
+        <v>40.32</v>
       </c>
     </row>
     <row r="36">
@@ -1244,13 +1287,13 @@
         </is>
       </c>
       <c r="B39" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" t="n">
         <v>5</v>
       </c>
-      <c r="C39" t="n">
-        <v>4</v>
-      </c>
       <c r="D39" t="n">
-        <v>148.14</v>
+        <v>151.18</v>
       </c>
     </row>
     <row r="40">
@@ -1371,213 +1414,229 @@
         <v>-10.98</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3.04</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>108.61</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>66.70999999999999</v>
+        <v>108.61</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>66.70999999999999</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>0.60–0.62</t>
         </is>
       </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" t="n">
-        <v>-10.98</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-7.94</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
-        <v>108.61</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>23.67</v>
+        <v>108.61</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" t="n">
-        <v>10.5</v>
+        <v>23.67</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>13.54</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>0.20%+</t>
         </is>
       </c>
-      <c r="B58" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" t="n">
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
         <v>21.56</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>4</v>
-      </c>
-      <c r="C61" t="n">
-        <v>3</v>
-      </c>
-      <c r="D61" t="n">
-        <v>37.28</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" t="n">
+        <v>40.32</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B62" t="n">
+      <c r="B63" t="n">
         <v>2</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C63" t="n">
         <v>2</v>
       </c>
-      <c r="D62" t="n">
+      <c r="D63" t="n">
         <v>127.06</v>
       </c>
     </row>

</xml_diff>